<commit_message>
DRA 1.6.1, JGA 1.3.1
</commit_message>
<xml_diff>
--- a/example/JSUB999999_jga_metadata.xlsx
+++ b/example/JSUB999999_jga_metadata.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8C7669-DD6D-4CAD-A322-F2BB99340D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4EC1BA-52F4-4C82-BF20-E8DDC56C8B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="906" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="12" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="919">
   <si>
     <t>E-mail</t>
     <phoneticPr fontId="1"/>
@@ -4585,7 +4585,46 @@
     <t>Sentosa SQ301</t>
   </si>
   <si>
+    <t>Illumina MiSeq i100</t>
+  </si>
+  <si>
+    <t>Illumina MiSeq i100 Plus</t>
+  </si>
+  <si>
     <t>Illumina NovaSeq X Plus</t>
+  </si>
+  <si>
+    <t>DNBSEQ-T1+</t>
+  </si>
+  <si>
+    <t>CycloneSEQ</t>
+  </si>
+  <si>
+    <t>SURFSeq 5000</t>
+  </si>
+  <si>
+    <t>SURFSeq Q</t>
+  </si>
+  <si>
+    <t>Saluseq Nimbo</t>
+  </si>
+  <si>
+    <t>Salus Pro</t>
+  </si>
+  <si>
+    <t>Salus EVO</t>
+  </si>
+  <si>
+    <t>G-seq500</t>
+  </si>
+  <si>
+    <t>G4</t>
+  </si>
+  <si>
+    <t>JGA xsd 1.3.1 に対応</t>
+    <rPh sb="15" eb="17">
+      <t>タイオウ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -5146,7 +5185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="126.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -5273,7 +5312,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A28" s="7">
-        <v>45953</v>
+        <v>46077</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.5">
@@ -5423,6 +5462,14 @@
       </c>
       <c r="B48" s="7">
         <v>45953</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A49" s="1" t="s">
+        <v>918</v>
+      </c>
+      <c r="B49" s="7">
+        <v>46077</v>
       </c>
     </row>
   </sheetData>
@@ -5443,7 +5490,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="28.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -5987,7 +6034,7 @@
         <v>241</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>886</v>
+        <v>906</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>663</v>
@@ -6010,7 +6057,7 @@
         <v>242</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>887</v>
+        <v>907</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>288</v>
@@ -6027,7 +6074,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B18" s="1" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>289</v>
@@ -6044,7 +6091,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B19" s="1" t="s">
-        <v>906</v>
+        <v>887</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>664</v>
@@ -6061,7 +6108,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B20" s="1" t="s">
-        <v>637</v>
+        <v>888</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>290</v>
@@ -6078,7 +6125,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B21" s="1" t="s">
-        <v>638</v>
+        <v>908</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>291</v>
@@ -6095,7 +6142,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B22" s="1" t="s">
-        <v>735</v>
+        <v>637</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>665</v>
@@ -6112,7 +6159,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B23" s="1" t="s">
-        <v>736</v>
+        <v>638</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>292</v>
@@ -6129,7 +6176,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B24" s="1" t="s">
-        <v>889</v>
+        <v>735</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>293</v>
@@ -6146,7 +6193,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B25" s="1" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>294</v>
@@ -6163,7 +6210,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B26" s="1" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>295</v>
@@ -6180,7 +6227,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B27" s="1" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>296</v>
@@ -6197,7 +6244,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B28" s="1" t="s">
-        <v>732</v>
+        <v>890</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>297</v>
@@ -6211,7 +6258,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B29" s="1" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>298</v>
@@ -6225,7 +6272,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B30" s="1" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>299</v>
@@ -6239,7 +6286,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B31" s="1" t="s">
-        <v>891</v>
+        <v>909</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>270</v>
@@ -6253,7 +6300,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.5">
       <c r="B32" s="1" t="s">
-        <v>267</v>
+        <v>729</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>740</v>
@@ -6264,7 +6311,7 @@
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B33" s="1" t="s">
-        <v>645</v>
+        <v>734</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>325</v>
@@ -6275,7 +6322,7 @@
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B34" s="1" t="s">
-        <v>646</v>
+        <v>891</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>326</v>
@@ -6286,7 +6333,7 @@
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B35" s="1" t="s">
-        <v>733</v>
+        <v>910</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>660</v>
@@ -6297,7 +6344,7 @@
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B36" s="1" t="s">
-        <v>892</v>
+        <v>267</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>658</v>
@@ -6308,7 +6355,7 @@
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B37" s="1" t="s">
-        <v>893</v>
+        <v>645</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>659</v>
@@ -6319,7 +6366,7 @@
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B38" s="1" t="s">
-        <v>894</v>
+        <v>646</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>277</v>
@@ -6330,7 +6377,7 @@
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B39" s="1" t="s">
-        <v>642</v>
+        <v>733</v>
       </c>
       <c r="K39" s="1" t="s">
         <v>394</v>
@@ -6338,7 +6385,7 @@
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B40" s="1" t="s">
-        <v>643</v>
+        <v>892</v>
       </c>
       <c r="K40" s="1" t="s">
         <v>395</v>
@@ -6346,7 +6393,7 @@
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B41" s="1" t="s">
-        <v>644</v>
+        <v>893</v>
       </c>
       <c r="K41" s="1" t="s">
         <v>396</v>
@@ -6354,7 +6401,7 @@
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B42" s="1" t="s">
-        <v>737</v>
+        <v>894</v>
       </c>
       <c r="K42" s="1" t="s">
         <v>693</v>
@@ -6362,7 +6409,7 @@
     </row>
     <row r="43" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B43" s="1" t="s">
-        <v>738</v>
+        <v>642</v>
       </c>
       <c r="K43" s="1" t="s">
         <v>397</v>
@@ -6370,7 +6417,7 @@
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B44" s="1" t="s">
-        <v>739</v>
+        <v>643</v>
       </c>
       <c r="K44" s="1" t="s">
         <v>694</v>
@@ -6378,7 +6425,7 @@
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B45" s="1" t="s">
-        <v>268</v>
+        <v>644</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>752</v>
@@ -6386,7 +6433,7 @@
     </row>
     <row r="46" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B46" s="1" t="s">
-        <v>269</v>
+        <v>737</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>753</v>
@@ -6394,7 +6441,7 @@
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B47" s="1" t="s">
-        <v>895</v>
+        <v>738</v>
       </c>
       <c r="K47" s="1" t="s">
         <v>754</v>
@@ -6402,7 +6449,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B48" s="1" t="s">
-        <v>896</v>
+        <v>739</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>695</v>
@@ -6410,7 +6457,7 @@
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B49" s="1" t="s">
-        <v>897</v>
+        <v>268</v>
       </c>
       <c r="K49" s="1" t="s">
         <v>696</v>
@@ -6418,7 +6465,7 @@
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B50" s="1" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
       <c r="K50" s="1" t="s">
         <v>697</v>
@@ -6426,7 +6473,7 @@
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B51" s="1" t="s">
-        <v>245</v>
+        <v>895</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>698</v>
@@ -6434,7 +6481,7 @@
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B52" s="1" t="s">
-        <v>246</v>
+        <v>896</v>
       </c>
       <c r="K52" s="1" t="s">
         <v>299</v>
@@ -6442,156 +6489,211 @@
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B53" s="1" t="s">
-        <v>247</v>
+        <v>897</v>
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B54" s="1" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B55" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B56" s="1" t="s">
-        <v>647</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B57" s="1" t="s">
-        <v>648</v>
+        <v>247</v>
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B58" s="1" t="s">
-        <v>649</v>
+        <v>248</v>
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B59" s="1" t="s">
-        <v>650</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B60" s="1" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B61" s="1" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B62" s="1" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B63" s="1" t="s">
-        <v>898</v>
+        <v>650</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.5">
       <c r="B64" s="1" t="s">
-        <v>899</v>
+        <v>651</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B65" s="1" t="s">
-        <v>900</v>
+        <v>652</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B66" s="1" t="s">
-        <v>901</v>
+        <v>653</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B67" s="1" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B68" s="1" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B69" s="1" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B70" s="1" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B71" s="1" t="s">
-        <v>259</v>
+        <v>912</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B72" s="1" t="s">
-        <v>260</v>
+        <v>901</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B73" s="1" t="s">
-        <v>261</v>
+        <v>902</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B74" s="1" t="s">
-        <v>262</v>
+        <v>903</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B75" s="1" t="s">
-        <v>263</v>
+        <v>904</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B76" s="1" t="s">
-        <v>264</v>
+        <v>905</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B77" s="1" t="s">
-        <v>265</v>
+        <v>913</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B78" s="1" t="s">
-        <v>639</v>
+        <v>914</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B79" s="1" t="s">
-        <v>640</v>
+        <v>915</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B80" s="1" t="s">
-        <v>641</v>
+        <v>916</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B81" s="1" t="s">
-        <v>258</v>
+        <v>917</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B82" s="1" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.5">
       <c r="B83" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B84" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B85" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B86" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B87" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B88" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B89" s="1" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B90" s="1" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B91" s="1" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B92" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B93" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.5">
+      <c r="B94" s="1" t="s">
         <v>270</v>
       </c>
     </row>
@@ -9419,7 +9521,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000006000000}">
           <x14:formula1>
-            <xm:f>Admin!$B$2:$B$83</xm:f>
+            <xm:f>Admin!$B$2:$B$94</xm:f>
           </x14:formula1>
           <xm:sqref>H4:H103 H3</xm:sqref>
         </x14:dataValidation>

</xml_diff>